<commit_message>
Maj ObservationRepas pour utiliser extension ParticipantPresent e3443274417d576cff775f48bb5a3bc5fec58204
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-encounter-evenement.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-encounter-evenement.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-11T13:38:26+00:00</t>
+    <t>2026-06-12T07:33:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1908,7 +1908,9 @@
     <t>Indique la présence du participant lors de l'événement.</t>
   </si>
   <si>
-    <t>Indique la présence du participant à l'événement.</t>
+    <t>Indique la présence du participant à l'événement.
+Evènement : Indique la présence du participant à l'événement.
+Repas : Indique la présence de l'usager au repas.</t>
   </si>
   <si>
     <t>Participant.presenceParticipant</t>

</xml_diff>

<commit_message>
fix slicing mapping 4a1d72f3bfda750a014f3c9151e9bc2a760b76c1
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-encounter-evenement.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-encounter-evenement.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-12T07:33:45+00:00</t>
+    <t>2026-06-12T07:50:14+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -927,8 +927,7 @@
   </si>
   <si>
     <t xml:space="preserve">
-- **Événement** : évènement nécessitant ou non la présence physique de l’usager.
-- **Repas** : Présence de l'usager au repas.</t>
+- **Événement** : évènement nécessitant ou non la présence physique de l’usager.</t>
   </si>
   <si>
     <t>usagerPresent</t>
@@ -1909,8 +1908,8 @@
   </si>
   <si>
     <t>Indique la présence du participant à l'événement.
-Evènement : Indique la présence du participant à l'événement.
-Repas : Indique la présence de l'usager au repas.</t>
+- **Événement** :Indique la présence du participant à l'événement.
+- **Repas** : Indique la présence de l'usager au repas.</t>
   </si>
   <si>
     <t>Participant.presenceParticipant</t>

</xml_diff>